<commit_message>
Met en valeur les onglets Philosophes/Courants sur la page recherche
Les boutons de type deviennent des onglets proeminents (bordure, style
actif marque) plutot que de simples petits boutons. En mode Courants,
le bloc Occidental/Oriental est immediatement visible et mis en avant
(encadre, boutons plus grands, label "Tradition") sans clic supplementaire.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-modernes.xlsx
+++ b/data/frise-philosophes-modernes.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="754">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="763">
   <si>
     <t xml:space="preserve">FRISE DES PHILOSOPHES MODERNES (AUTRES) — Données source</t>
   </si>
@@ -1162,7 +1162,7 @@
     <t xml:space="preserve">ethique ; epistemologie</t>
   </si>
   <si>
-    <t xml:space="preserve">Analytique ; Intuitionnisme</t>
+    <t xml:space="preserve">Analytique ; Intuitionnisme ; Cognitivisme</t>
   </si>
   <si>
     <t xml:space="preserve">philosophe anglais connu pour son parti pris contre le sophisme naturaliste.</t>
@@ -1959,6 +1959,34 @@
   </si>
   <si>
     <t xml:space="preserve">philosophe espagnol intègrant l'agnosticisme dans une réflexion éthique et religieuse évolutive.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1910 – 1989</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alfred Jules AYER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Alfred_Jules_Ayer" title=" Wikipedia"&gt;Alfred Jules AYER&lt;/a&gt; souvent surnommé « Freddie », était un philosophe britannique qui a joué un rôle central dans la diffusion du positivisme logique dans le monde anglophone. Né à Londres dans une famille d’origine suisse et néerlandaise, il fait ses études à Eton puis à Oxford, où il devient rapidement  &lt;a href="https://www.la-philosophie.fr/philosophie-analytique/alfred-jules-ayer-8.html"  title="philosophie analytique par la philosophie"&gt; une figure majeure &lt;/a&gt; de la philosophie analytique. C’est à seulement 24 ans qu’il publie son ouvrage le plus célèbre, Language, Truth, and Logic (1936), qui expose avec clarté et rigueur les thèses fondamentales du Cercle de Vienne et établit sa réputation internationale. &lt;/p&gt; &lt;p&gt; Au cœur de sa philosophie se trouve le principe de vérification, selon lequel une proposition n’a de sens cognitif que si elle est soit analytique (vraie en vertu de la signification des termes, comme en logique ou en mathématiques), soit empiriquement vérifiable (c’est-à-dire susceptible d’être confirmée ou infirmée par l’expérience). Ce critère lui permet de rejeter comme dénuées de sens littéral la plupart des affirmations de la métaphysique traditionnelle, de la théologie spéculative et de certaines formes d’éthique normative : elles ne sont pas fausses, mais simplement non vérifiables, donc dépourvues de contenu factuel. Il distingue ainsi strictement la philosophie, conçue comme analyse logique du langage, des sciences empiriques, seules habilitées à produire des connaissances sur le monde. &lt;/p&gt; &lt;p&gt; En éthique, il défend une position connue sous  &lt;a href="https://www.youtube.com/watch?v=HG5kIR6iF8g"  title="A,J, Ayer’s Emotivism par philosophy Vibe"&gt;le nom d’émotivisme. &lt;/a&gt;  Selon lui, les jugements moraux (« Le vol est mal », « La générosité est bonne ») n’expriment pas des faits objectifs, car il n’existe pas de « faits moraux » vérifiables empiriquement. Ils sont plutôt l’expression d’attitudes émotionnelles ou de prescriptions destinées à influencer les comportements d’autrui. Cette thèse s’inscrit dans une distinction radicale entre faits et valeurs : la science et la logique peuvent traiter des premiers, mais les secondes relèvent de la subjectivité et ne peuvent fonder aucune connaissance objective. &lt;/p&gt; &lt;p&gt; Au fil de sa carrière, il a nuancé certaines de ses positions initiales, notamment en reformulant le principe de vérification pour répondre aux objections (par exemple, en distinguant vérification directe et indirecte). Il a aussi évolué sur des questions de perception, de causalité et de liberté, tout en restant fidèle à un empirisme rigoureux et à une méfiance envers toute forme de métaphysique spéculative. Malgré les critiques ultérieures adressées au positivisme logique — notamment sur le statut même du principe de vérification —, son influence sur la philosophie analytique du XXᵉ siècle reste profonde, en particulier dans les débats sur le sens, la connaissance et l’éthique. &lt;/p&gt; 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-XYuh39J-zo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A,J, Ayer par ThamesTv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.laphilo.fr/pho/ajayer-mini.webp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethique ; logique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positivisme logique ; Analytique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">philosophe britannique qui a joué un rôle central dans la diffusion du positivisme logique dans le monde anglophone.</t>
   </si>
   <si>
     <t xml:space="preserve">1960</t>
@@ -3106,7 +3134,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M91"/>
+  <dimension ref="A1:M92"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.34"/>
@@ -5597,7 +5625,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="136.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="173.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="n">
         <v>1909</v>
       </c>
@@ -5636,90 +5664,90 @@
         <v>569</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="136.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="351.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="n">
-        <v>1911</v>
-      </c>
-      <c r="B67" s="7" t="s">
+        <v>1910</v>
+      </c>
+      <c r="B67" s="7" t="n">
+        <v>1989</v>
+      </c>
+      <c r="C67" s="7" t="s">
         <v>570</v>
       </c>
-      <c r="C67" s="7" t="s">
+      <c r="D67" s="8" t="s">
         <v>571</v>
       </c>
-      <c r="D67" s="8" t="s">
+      <c r="E67" s="11" t="s">
         <v>572</v>
       </c>
-      <c r="E67" s="12" t="s">
+      <c r="F67" s="7" t="s">
         <v>573</v>
       </c>
-      <c r="F67" s="7" t="s">
+      <c r="G67" s="9" t="s">
         <v>574</v>
       </c>
-      <c r="G67" s="9" t="s">
+      <c r="H67" s="10" t="s">
         <v>575</v>
-      </c>
-      <c r="H67" s="10" t="s">
-        <v>576</v>
       </c>
       <c r="I67" s="9"/>
       <c r="J67" s="2" t="s">
         <v>33</v>
       </c>
       <c r="K67" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="L67" s="2" t="s">
         <v>577</v>
       </c>
-      <c r="L67" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="M67" s="2" t="s">
+      <c r="M67" s="14" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="306.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="n">
         <v>1911</v>
       </c>
-      <c r="B68" s="7" t="n">
-        <v>1995</v>
+      <c r="B68" s="7" t="s">
+        <v>579</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>580</v>
-      </c>
-      <c r="E68" s="11" t="s">
         <v>581</v>
       </c>
+      <c r="E68" s="12" t="s">
+        <v>582</v>
+      </c>
       <c r="F68" s="7" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="H68" s="10" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="I68" s="9"/>
       <c r="J68" s="2" t="s">
-        <v>448</v>
+        <v>33</v>
       </c>
       <c r="K68" s="2" t="s">
-        <v>151</v>
+        <v>586</v>
       </c>
       <c r="L68" s="2" t="s">
-        <v>585</v>
+        <v>94</v>
       </c>
       <c r="M68" s="2" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="255.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="n">
-        <v>1913</v>
-      </c>
-      <c r="B69" s="7" t="s">
-        <v>587</v>
+        <v>1911</v>
+      </c>
+      <c r="B69" s="7" t="n">
+        <v>1995</v>
       </c>
       <c r="C69" s="7" t="s">
         <v>588</v>
@@ -5727,7 +5755,7 @@
       <c r="D69" s="8" t="s">
         <v>589</v>
       </c>
-      <c r="E69" s="12" t="s">
+      <c r="E69" s="11" t="s">
         <v>590</v>
       </c>
       <c r="F69" s="7" t="s">
@@ -5741,49 +5769,49 @@
       </c>
       <c r="I69" s="9"/>
       <c r="J69" s="2" t="s">
-        <v>33</v>
+        <v>448</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>577</v>
+        <v>151</v>
       </c>
       <c r="L69" s="2" t="s">
-        <v>94</v>
+        <v>594</v>
       </c>
       <c r="M69" s="2" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="179.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="n">
-        <v>1914</v>
+        <v>1913</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="D70" s="8" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="E70" s="12" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="F70" s="7" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>600</v>
-      </c>
-      <c r="H70" s="9" t="s">
         <v>601</v>
+      </c>
+      <c r="H70" s="10" t="s">
+        <v>602</v>
       </c>
       <c r="I70" s="9"/>
       <c r="J70" s="2" t="s">
-        <v>602</v>
+        <v>33</v>
       </c>
       <c r="K70" s="2" t="s">
-        <v>180</v>
+        <v>586</v>
       </c>
       <c r="L70" s="2" t="s">
         <v>94</v>
@@ -5792,75 +5820,75 @@
         <v>603</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="314.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="1" t="n">
+    <row r="71" customFormat="false" ht="179.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="7" t="n">
+        <v>1914</v>
+      </c>
+      <c r="B71" s="7" t="s">
+        <v>604</v>
+      </c>
+      <c r="C71" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="D71" s="8" t="s">
+        <v>606</v>
+      </c>
+      <c r="E71" s="12" t="s">
+        <v>607</v>
+      </c>
+      <c r="F71" s="7" t="s">
+        <v>608</v>
+      </c>
+      <c r="G71" s="9" t="s">
+        <v>609</v>
+      </c>
+      <c r="H71" s="9" t="s">
+        <v>610</v>
+      </c>
+      <c r="I71" s="9"/>
+      <c r="J71" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="K71" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="L71" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="M71" s="2" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="314.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="n">
         <v>1919</v>
       </c>
-      <c r="B71" s="1" t="n">
+      <c r="B72" s="1" t="n">
         <v>2001</v>
       </c>
-      <c r="C71" s="1" t="s">
-        <v>604</v>
-      </c>
-      <c r="D71" s="1" t="s">
-        <v>605</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>606</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>607</v>
-      </c>
-      <c r="G71" s="2" t="s">
-        <v>608</v>
-      </c>
-      <c r="H71" s="2" t="s">
-        <v>609</v>
-      </c>
-      <c r="J71" s="2" t="s">
+      <c r="C72" s="1" t="s">
+        <v>613</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>614</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>616</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="J72" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K71" s="2" t="s">
+      <c r="K72" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="L71" s="2" t="s">
-        <v>610</v>
-      </c>
-      <c r="M71" s="2" t="s">
-        <v>611</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="164.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="7" t="n">
-        <v>1922</v>
-      </c>
-      <c r="B72" s="7" t="s">
-        <v>546</v>
-      </c>
-      <c r="C72" s="7" t="s">
-        <v>612</v>
-      </c>
-      <c r="D72" s="8" t="s">
-        <v>613</v>
-      </c>
-      <c r="E72" s="11" t="s">
-        <v>614</v>
-      </c>
-      <c r="F72" s="7" t="s">
-        <v>615</v>
-      </c>
-      <c r="G72" s="9" t="s">
-        <v>616</v>
-      </c>
-      <c r="H72" s="9" t="s">
-        <v>617</v>
-      </c>
-      <c r="I72" s="9"/>
-      <c r="J72" s="2" t="s">
-        <v>618</v>
-      </c>
-      <c r="K72" s="2" t="s">
-        <v>170</v>
       </c>
       <c r="L72" s="2" t="s">
         <v>619</v>
@@ -5869,69 +5897,69 @@
         <v>620</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="164.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="n">
         <v>1922</v>
       </c>
       <c r="B73" s="7" t="s">
+        <v>546</v>
+      </c>
+      <c r="C73" s="7" t="s">
         <v>621</v>
       </c>
-      <c r="C73" s="7" t="s">
+      <c r="D73" s="8" t="s">
         <v>622</v>
       </c>
-      <c r="D73" s="8" t="s">
+      <c r="E73" s="11" t="s">
         <v>623</v>
       </c>
-      <c r="E73" s="11" t="s">
+      <c r="F73" s="7" t="s">
         <v>624</v>
       </c>
-      <c r="F73" s="7" t="s">
+      <c r="G73" s="9" t="s">
         <v>625</v>
       </c>
-      <c r="G73" s="9" t="s">
+      <c r="H73" s="9" t="s">
         <v>626</v>
-      </c>
-      <c r="H73" s="9" t="s">
-        <v>627</v>
       </c>
       <c r="I73" s="9"/>
       <c r="J73" s="2" t="s">
-        <v>33</v>
+        <v>627</v>
       </c>
       <c r="K73" s="2" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="L73" s="2" t="s">
-        <v>94</v>
+        <v>628</v>
       </c>
       <c r="M73" s="2" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="158.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="n">
-        <v>1923</v>
+        <v>1922</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>631</v>
-      </c>
-      <c r="E74" s="10" t="s">
         <v>632</v>
       </c>
+      <c r="E74" s="11" t="s">
+        <v>633</v>
+      </c>
       <c r="F74" s="7" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="G74" s="9" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="I74" s="9"/>
       <c r="J74" s="2" t="s">
@@ -5944,132 +5972,130 @@
         <v>94</v>
       </c>
       <c r="M74" s="2" t="s">
-        <v>636</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="123.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="158.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="n">
-        <v>1924</v>
-      </c>
-      <c r="B75" s="7" t="n">
-        <v>2019</v>
+        <v>1923</v>
+      </c>
+      <c r="B75" s="7" t="s">
+        <v>638</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="D75" s="8" t="s">
-        <v>638</v>
-      </c>
-      <c r="E75" s="11" t="s">
-        <v>639</v>
+        <v>640</v>
+      </c>
+      <c r="E75" s="10" t="s">
+        <v>641</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>641</v>
-      </c>
-      <c r="H75" s="10" t="s">
-        <v>642</v>
+        <v>643</v>
+      </c>
+      <c r="H75" s="9" t="s">
+        <v>644</v>
       </c>
       <c r="I75" s="9"/>
       <c r="J75" s="2" t="s">
         <v>33</v>
       </c>
       <c r="K75" s="2" t="s">
-        <v>312</v>
+        <v>180</v>
       </c>
       <c r="L75" s="2" t="s">
         <v>94</v>
       </c>
       <c r="M75" s="2" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="183" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="123.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="n">
         <v>1924</v>
       </c>
       <c r="B76" s="7" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>646</v>
+      </c>
+      <c r="D76" s="8" t="s">
+        <v>647</v>
+      </c>
+      <c r="E76" s="11" t="s">
+        <v>648</v>
+      </c>
+      <c r="F76" s="7" t="s">
+        <v>649</v>
+      </c>
+      <c r="G76" s="9" t="s">
+        <v>650</v>
+      </c>
+      <c r="H76" s="10" t="s">
+        <v>651</v>
+      </c>
+      <c r="I76" s="9"/>
+      <c r="J76" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K76" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="L76" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="M76" s="2" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="183" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="7" t="n">
+        <v>1924</v>
+      </c>
+      <c r="B77" s="7" t="n">
         <v>2003</v>
       </c>
-      <c r="C76" s="7" t="s">
-        <v>644</v>
-      </c>
-      <c r="D76" s="8" t="s">
-        <v>645</v>
-      </c>
-      <c r="E76" s="11" t="s">
-        <v>646</v>
-      </c>
-      <c r="F76" s="7"/>
-      <c r="G76" s="9"/>
-      <c r="H76" s="10" t="s">
-        <v>647</v>
-      </c>
-      <c r="I76" s="10" t="s">
-        <v>648</v>
-      </c>
-      <c r="J76" s="2" t="s">
+      <c r="C77" s="7" t="s">
+        <v>653</v>
+      </c>
+      <c r="D77" s="8" t="s">
+        <v>654</v>
+      </c>
+      <c r="E77" s="11" t="s">
+        <v>655</v>
+      </c>
+      <c r="F77" s="7"/>
+      <c r="G77" s="9"/>
+      <c r="H77" s="10" t="s">
+        <v>656</v>
+      </c>
+      <c r="I77" s="10" t="s">
+        <v>657</v>
+      </c>
+      <c r="J77" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="K76" s="2" t="s">
-        <v>649</v>
-      </c>
-      <c r="L76" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="M76" s="14" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="339" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="7" t="n">
-        <v>1925</v>
-      </c>
-      <c r="B77" s="7" t="s">
-        <v>629</v>
-      </c>
-      <c r="C77" s="7" t="s">
-        <v>652</v>
-      </c>
-      <c r="D77" s="8" t="s">
-        <v>653</v>
-      </c>
-      <c r="E77" s="11" t="s">
-        <v>654</v>
-      </c>
-      <c r="F77" s="7" t="s">
-        <v>655</v>
-      </c>
-      <c r="G77" s="9" t="s">
-        <v>656</v>
-      </c>
-      <c r="H77" s="10" t="s">
-        <v>657</v>
-      </c>
-      <c r="I77" s="10" t="s">
+      <c r="K77" s="2" t="s">
         <v>658</v>
       </c>
-      <c r="J77" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="K77" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="L77" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="M77" s="2" t="s">
         <v>659</v>
       </c>
-    </row>
-    <row r="78" customFormat="false" ht="272.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M77" s="14" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="339" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="n">
         <v>1925</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>660</v>
+        <v>638</v>
       </c>
       <c r="C78" s="7" t="s">
         <v>661</v>
@@ -6077,7 +6103,7 @@
       <c r="D78" s="8" t="s">
         <v>662</v>
       </c>
-      <c r="E78" s="12" t="s">
+      <c r="E78" s="11" t="s">
         <v>663</v>
       </c>
       <c r="F78" s="7" t="s">
@@ -6086,26 +6112,28 @@
       <c r="G78" s="9" t="s">
         <v>665</v>
       </c>
-      <c r="H78" s="9" t="s">
+      <c r="H78" s="10" t="s">
         <v>666</v>
       </c>
-      <c r="I78" s="9"/>
+      <c r="I78" s="10" t="s">
+        <v>667</v>
+      </c>
       <c r="J78" s="2" t="s">
-        <v>294</v>
+        <v>33</v>
       </c>
       <c r="K78" s="2" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="L78" s="2" t="s">
-        <v>667</v>
-      </c>
-      <c r="M78" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="M78" s="2" t="s">
         <v>668</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="267.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="272.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="n">
-        <v>1926</v>
+        <v>1925</v>
       </c>
       <c r="B79" s="7" t="s">
         <v>669</v>
@@ -6116,7 +6144,7 @@
       <c r="D79" s="8" t="s">
         <v>671</v>
       </c>
-      <c r="E79" s="9" t="s">
+      <c r="E79" s="12" t="s">
         <v>672</v>
       </c>
       <c r="F79" s="7" t="s">
@@ -6130,7 +6158,7 @@
       </c>
       <c r="I79" s="9"/>
       <c r="J79" s="2" t="s">
-        <v>22</v>
+        <v>294</v>
       </c>
       <c r="K79" s="2" t="s">
         <v>65</v>
@@ -6138,118 +6166,118 @@
       <c r="L79" s="2" t="s">
         <v>676</v>
       </c>
-      <c r="M79" s="2" t="s">
+      <c r="M79" s="14" t="s">
         <v>677</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="358.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="1" t="n">
+    <row r="80" customFormat="false" ht="267.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="7" t="n">
         <v>1926</v>
       </c>
-      <c r="B80" s="1" t="n">
+      <c r="B80" s="7" t="s">
+        <v>678</v>
+      </c>
+      <c r="C80" s="7" t="s">
+        <v>679</v>
+      </c>
+      <c r="D80" s="8" t="s">
+        <v>680</v>
+      </c>
+      <c r="E80" s="9" t="s">
+        <v>681</v>
+      </c>
+      <c r="F80" s="7" t="s">
+        <v>682</v>
+      </c>
+      <c r="G80" s="9" t="s">
+        <v>683</v>
+      </c>
+      <c r="H80" s="9" t="s">
+        <v>684</v>
+      </c>
+      <c r="I80" s="9"/>
+      <c r="J80" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K80" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L80" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="M80" s="2" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="358.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="1" t="n">
+        <v>1926</v>
+      </c>
+      <c r="B81" s="1" t="n">
         <v>2002</v>
       </c>
-      <c r="C80" s="1" t="s">
-        <v>670</v>
-      </c>
-      <c r="D80" s="1" t="s">
-        <v>678</v>
-      </c>
-      <c r="E80" s="2" t="s">
+      <c r="C81" s="1" t="s">
         <v>679</v>
       </c>
-      <c r="F80" s="1" t="s">
-        <v>680</v>
-      </c>
-      <c r="G80" s="2" t="s">
-        <v>681</v>
-      </c>
-      <c r="H80" s="2" t="s">
-        <v>682</v>
-      </c>
-      <c r="J80" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="K80" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L80" s="2" t="s">
-        <v>683</v>
-      </c>
-      <c r="M80" s="2" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="7" t="n">
-        <v>1929</v>
-      </c>
-      <c r="B81" s="7" t="s">
-        <v>685</v>
-      </c>
-      <c r="C81" s="7" t="s">
-        <v>686</v>
-      </c>
-      <c r="D81" s="8" t="s">
+      <c r="D81" s="1" t="s">
         <v>687</v>
       </c>
-      <c r="E81" s="13" t="s">
+      <c r="E81" s="2" t="s">
         <v>688</v>
       </c>
-      <c r="F81" s="7" t="s">
+      <c r="F81" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="G81" s="9" t="s">
+      <c r="G81" s="2" t="s">
         <v>690</v>
       </c>
-      <c r="H81" s="9" t="s">
+      <c r="H81" s="2" t="s">
         <v>691</v>
       </c>
-      <c r="I81" s="9"/>
       <c r="J81" s="2" t="s">
         <v>33</v>
       </c>
       <c r="K81" s="2" t="s">
-        <v>205</v>
+        <v>74</v>
       </c>
       <c r="L81" s="2" t="s">
-        <v>94</v>
+        <v>692</v>
       </c>
       <c r="M81" s="2" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="117.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="n">
         <v>1929</v>
       </c>
       <c r="B82" s="7" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="D82" s="8" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="E82" s="13" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="F82" s="7" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="G82" s="9" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="H82" s="9" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="I82" s="9"/>
       <c r="J82" s="2" t="s">
         <v>33</v>
       </c>
       <c r="K82" s="2" t="s">
-        <v>700</v>
+        <v>205</v>
       </c>
       <c r="L82" s="2" t="s">
         <v>94</v>
@@ -6258,9 +6286,9 @@
         <v>701</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="101.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="117.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="n">
-        <v>1930</v>
+        <v>1929</v>
       </c>
       <c r="B83" s="7" t="s">
         <v>702</v>
@@ -6271,7 +6299,7 @@
       <c r="D83" s="8" t="s">
         <v>704</v>
       </c>
-      <c r="E83" s="11" t="s">
+      <c r="E83" s="13" t="s">
         <v>705</v>
       </c>
       <c r="F83" s="7" t="s">
@@ -6288,91 +6316,91 @@
         <v>33</v>
       </c>
       <c r="K83" s="2" t="s">
-        <v>180</v>
+        <v>709</v>
       </c>
       <c r="L83" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="84" customFormat="false" ht="183" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M83" s="2" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="101.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="n">
-        <v>1933</v>
-      </c>
-      <c r="B84" s="7" t="n">
-        <v>2018</v>
+        <v>1930</v>
+      </c>
+      <c r="B84" s="7" t="s">
+        <v>711</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="D84" s="8" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="E84" s="11" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="F84" s="7" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="G84" s="9" t="s">
-        <v>713</v>
-      </c>
-      <c r="H84" s="10" t="s">
-        <v>714</v>
+        <v>716</v>
+      </c>
+      <c r="H84" s="9" t="s">
+        <v>717</v>
       </c>
       <c r="I84" s="9"/>
       <c r="J84" s="2" t="s">
-        <v>448</v>
+        <v>33</v>
       </c>
       <c r="K84" s="2" t="s">
-        <v>74</v>
+        <v>180</v>
       </c>
       <c r="L84" s="2" t="s">
-        <v>715</v>
-      </c>
-      <c r="M84" s="14" t="s">
-        <v>716</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="333.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="183" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="n">
-        <v>1934</v>
+        <v>1933</v>
       </c>
       <c r="B85" s="7" t="n">
-        <v>2026</v>
+        <v>2018</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="D85" s="8" t="s">
-        <v>718</v>
-      </c>
-      <c r="E85" s="12" t="s">
         <v>719</v>
       </c>
+      <c r="E85" s="11" t="s">
+        <v>720</v>
+      </c>
       <c r="F85" s="7" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="G85" s="9" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="H85" s="10" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="I85" s="9"/>
       <c r="J85" s="2" t="s">
-        <v>139</v>
+        <v>448</v>
       </c>
       <c r="K85" s="2" t="s">
-        <v>258</v>
+        <v>74</v>
       </c>
       <c r="L85" s="2" t="s">
-        <v>512</v>
-      </c>
-      <c r="M85" s="2" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="287.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>724</v>
+      </c>
+      <c r="M85" s="14" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="333.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="n">
         <v>1934</v>
       </c>
@@ -6380,164 +6408,193 @@
         <v>2026</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>717</v>
+        <v>726</v>
       </c>
       <c r="D86" s="8" t="s">
-        <v>724</v>
-      </c>
-      <c r="E86" s="11" t="s">
-        <v>725</v>
+        <v>727</v>
+      </c>
+      <c r="E86" s="12" t="s">
+        <v>728</v>
       </c>
       <c r="F86" s="7" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="G86" s="9" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="H86" s="10" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="I86" s="9"/>
       <c r="J86" s="2" t="s">
-        <v>511</v>
+        <v>139</v>
       </c>
       <c r="K86" s="2" t="s">
-        <v>74</v>
+        <v>258</v>
       </c>
       <c r="L86" s="2" t="s">
-        <v>729</v>
-      </c>
-      <c r="M86" s="14" t="s">
-        <v>730</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="217.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>512</v>
+      </c>
+      <c r="M86" s="2" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="287.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="n">
-        <v>1936</v>
+        <v>1934</v>
       </c>
       <c r="B87" s="7" t="n">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
       <c r="D87" s="8" t="s">
-        <v>732</v>
-      </c>
-      <c r="E87" s="13" t="s">
         <v>733</v>
       </c>
+      <c r="E87" s="11" t="s">
+        <v>734</v>
+      </c>
       <c r="F87" s="7" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="G87" s="9" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="H87" s="10" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="I87" s="9"/>
       <c r="J87" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="K87" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="L87" s="2" t="s">
+        <v>738</v>
+      </c>
+      <c r="M87" s="14" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="217.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A88" s="7" t="n">
+        <v>1936</v>
+      </c>
+      <c r="B88" s="7" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C88" s="7" t="s">
+        <v>740</v>
+      </c>
+      <c r="D88" s="8" t="s">
+        <v>741</v>
+      </c>
+      <c r="E88" s="13" t="s">
+        <v>742</v>
+      </c>
+      <c r="F88" s="7" t="s">
+        <v>743</v>
+      </c>
+      <c r="G88" s="9" t="s">
+        <v>744</v>
+      </c>
+      <c r="H88" s="10" t="s">
+        <v>745</v>
+      </c>
+      <c r="I88" s="9"/>
+      <c r="J88" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="K87" s="2" t="s">
+      <c r="K88" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="L87" s="2" t="s">
+      <c r="L88" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="M87" s="2" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="249" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="7" t="n">
-        <v>1942</v>
-      </c>
-      <c r="B88" s="7" t="s">
-        <v>660</v>
-      </c>
-      <c r="C88" s="7" t="s">
-        <v>738</v>
-      </c>
-      <c r="D88" s="8" t="s">
-        <v>739</v>
-      </c>
-      <c r="E88" s="10" t="s">
-        <v>740</v>
-      </c>
-      <c r="F88" s="7" t="s">
-        <v>741</v>
-      </c>
-      <c r="G88" s="9" t="s">
-        <v>742</v>
-      </c>
-      <c r="H88" s="10" t="s">
-        <v>743</v>
-      </c>
-      <c r="I88" s="10"/>
-      <c r="J88" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="K88" s="2" t="s">
-        <v>744</v>
-      </c>
-      <c r="L88" s="2" t="s">
-        <v>745</v>
       </c>
       <c r="M88" s="2" t="s">
         <v>746</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="61.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="1" t="n">
+    <row r="89" customFormat="false" ht="249" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A89" s="7" t="n">
+        <v>1942</v>
+      </c>
+      <c r="B89" s="7" t="s">
+        <v>669</v>
+      </c>
+      <c r="C89" s="7" t="s">
+        <v>747</v>
+      </c>
+      <c r="D89" s="8" t="s">
+        <v>748</v>
+      </c>
+      <c r="E89" s="10" t="s">
+        <v>749</v>
+      </c>
+      <c r="F89" s="7" t="s">
+        <v>750</v>
+      </c>
+      <c r="G89" s="9" t="s">
+        <v>751</v>
+      </c>
+      <c r="H89" s="10" t="s">
+        <v>752</v>
+      </c>
+      <c r="I89" s="10"/>
+      <c r="J89" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K89" s="2" t="s">
+        <v>753</v>
+      </c>
+      <c r="L89" s="2" t="s">
+        <v>754</v>
+      </c>
+      <c r="M89" s="2" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="61.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="1" t="n">
         <v>1954</v>
       </c>
-      <c r="B89" s="1" t="n">
+      <c r="B90" s="1" t="n">
         <v>2014</v>
       </c>
-      <c r="C89" s="1" t="s">
-        <v>747</v>
-      </c>
-      <c r="D89" s="1" t="s">
-        <v>748</v>
-      </c>
-      <c r="E89" s="14" t="s">
-        <v>749</v>
-      </c>
-      <c r="F89" s="1" t="s">
-        <v>750</v>
-      </c>
-      <c r="G89" s="2" t="s">
-        <v>751</v>
-      </c>
-      <c r="H89" s="2" t="s">
-        <v>752</v>
-      </c>
-      <c r="J89" s="2" t="s">
+      <c r="C90" s="1" t="s">
+        <v>756</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>757</v>
+      </c>
+      <c r="E90" s="14" t="s">
+        <v>758</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="G90" s="2" t="s">
+        <v>760</v>
+      </c>
+      <c r="H90" s="2" t="s">
+        <v>761</v>
+      </c>
+      <c r="J90" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="K89" s="2" t="s">
+      <c r="K90" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L89" s="2" t="s">
+      <c r="L90" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="M89" s="2" t="s">
-        <v>753</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="52.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E90" s="1"/>
-      <c r="G90" s="1"/>
-      <c r="H90" s="1"/>
-      <c r="I90" s="1"/>
-      <c r="J90" s="1"/>
-      <c r="K90" s="1"/>
-      <c r="L90" s="1"/>
-      <c r="M90" s="1"/>
-    </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M90" s="2" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="52.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E91" s="1"/>
       <c r="G91" s="1"/>
       <c r="H91" s="1"/>
@@ -6546,6 +6603,16 @@
       <c r="K91" s="1"/>
       <c r="L91" s="1"/>
       <c r="M91" s="1"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E92" s="1"/>
+      <c r="G92" s="1"/>
+      <c r="H92" s="1"/>
+      <c r="I92" s="1"/>
+      <c r="J92" s="1"/>
+      <c r="K92" s="1"/>
+      <c r="L92" s="1"/>
+      <c r="M92" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6612,26 +6679,28 @@
     <hyperlink ref="E65" r:id="rId57" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Eugenio_Garin&quot; title=&quot; Wikipedia&quot;&gt;Eugenio GARIN&lt;/a&gt;  fut un grand historien italien de la philosophie, surtout connu pour ses travaux sur la Renaissance et l’humanisme italien. Né à Rieti, il enseigna à Florence puis à l’École normale supérieure de Pise, et il a profondément renouvelé l’étude des idées en les replaçant toujours dans leur contexte historique. &lt;/p&gt; &lt;p&gt; Dans sa méthode, il refusait l’idée d’une vérité philosophique intemporelle et abstraite. Il défendait au contraire une lecture historique des œuvres, attentive aux rapports entre pensée, culture, politique et institutions, ce qui le rapprochait d’une attitude critique envers les certitudes absolues. &lt;/p&gt; &lt;p&gt; Son lien avec  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Agnosticisme&quot;  title=&quot; Agnosticisme  par Wikipedia&quot;&gt;L'agnosticisme &lt;/a&gt; n’est pas celui d’un fondateur ou d’un théoricien direct, mais plutôt celui d’un penseur qui a mis en avant la complexité, le doute et la diversité des positions humaines. Ses travaux sur l’humanisme montrent que la pensée de la Renaissance est traversée par des tensions entre savoir, foi, scepticisme et prudence intellectuelle. &lt;/p&gt; &lt;p&gt; On peut donc dire que Garin prolonge, d’une certaine manière, l’esprit de l’agnosticisme sans en faire un sujet central. Chez lui, l’essentiel est de comprendre comment les hommes pensent dans une époque donnée, plutôt que de chercher une réponse définitive aux grandes questions métaphysiques. &lt;/p&gt; "/>
     <hyperlink ref="E66" r:id="rId58" display="&lt;p&gt;&lt;a href=&quot;https://es.wikipedia.org/wiki/Jos%C3%A9_Luis_L%C3%B3pez_Aranguren&quot; title=&quot; Wikipedia&quot;&gt;José Luis Lopez ARANGUREN&lt;/a&gt;   philosophe et essayiste espagnol influent, intègre l'agnosticisme dans une réflexion éthique et religieuse évolutive, passant d'un catholicisme initial à une &quot;perplexité&quot; ouverte sur le doute. Né à Ávila, formé par Ortega y Gasset et Zubiri, il occupe la chaire d'éthique à l'Université Complutense de Madrid dès 1955. Catholique critique, il explore dans Catholicisme et protestantisme comme formes d'existence  les tensions entre foi et morale, influençant des disciples comme Muguerza. &lt;/p&gt; &lt;p&gt; Sans lien avec les origines historiques de  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Agnosticisme&quot;  title=&quot; Agnosticisme  par Wikipedia&quot;&gt;l'agnosticisme &lt;/a&gt;, il développe une &quot;éthique de la perplexité&quot; : refus des certitudes dogmatiques au profit d'une raison ouverte, dialoguant avec le protestantisme (Karl Barth) et la critique sociale. Exclu de l'université en 1965 pour contestation antifranquiste, il enseigne à Berkeley, nouant amitié avec Marcuse, et approfondit une pensée humaniste contre la technocratie. &lt;a href=&quot;https://www.youtube.com/watch?v=L3sJ7AvOT08&quot;  title=&quot; José Luis Aranguren  par Lecturas Fragmentadas&quot;&gt;Ses œuvres &lt;/a&gt; comme Ética (1958) et Propuestas morales (1985) lient morale, religion et politique sans absolutisme.https://www.athees.net/pourquoi-latheisme-et-pas-lagnosticisme/ &lt;/p&gt; &lt;p&gt; Sa position religieuse oscille : catholique &quot;progressiste&quot; puis laïc engagé, il valorise la dissidence intellectuelle et une &quot;justice sociale&quot; cosmopolite, écho à l'agnosticisme par son rejet des systèmes fermés. Penseur de la transition démocratique espagnole, il reçoit le Prix national d'essai (1989) et le Prince des Asturies (1995), léguant une philosophie de la solidarité humaniste. &lt;/p&gt;&#10;"/>
     <hyperlink ref="H66" r:id="rId59" display="https://laphilo.fr/pho/jlaranguren-mini.webp"/>
-    <hyperlink ref="H67" r:id="rId60" display="https://www.laphilo.fr/pho/jlaustin-mini.webp"/>
-    <hyperlink ref="H69" r:id="rId61" display="https://www.laphilo.fr/pho/pgrice-mini.webp"/>
-    <hyperlink ref="H71" r:id="rId62" display="https://www.laphilo.fr/pho/eanscombe-mini.webp"/>
-    <hyperlink ref="E73" r:id="rId63" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Stephen_Toulmin&quot;  title=&quot; Wikipedia&quot;&gt;Stephen TOULMIN&lt;/a&gt;  était un philosophe britanique  influencé par Wittgenstein, est un penseur majeur de la philosophie des sciences et de l'argumentation pratique. Né en Angleterre, il étudie à Cambridge, enseigne à Oxford, Leeds, puis aux États-Unis (notamment à Northwestern et USC). Critique du formalisme logique absolu, il prône une approche contextualisée des raisonnements, applicable au droit, à la médecine ou à la diplomatie, loin des abstractions syllogistiques. &lt;/p&gt; &lt;p&gt; Son œuvre fondatrice, The Uses of Argument (1958), introduit le  &lt;a href=&quot;https://www.youtube.com/watch?v=J1WDW2F-KBs&quot;  title=&quot; le modèle de Toulmin  par Mooc Cyu&quot;&gt;modèle d'argumentation de Toulmin &lt;/a&gt;  : une structure à six composantes pour analyser les débats réels. La claim (thèse), les grounds (données), le warrant (justification liant données et thèse), le backing (soutien du warrant), les qualifiers (modalisateurs comme &quot;probablement&quot;), et les rebuttals (contre-arguments). Ce schéma met en lumière les aspects &quot;field-dependent&quot; (dépendants du domaine) versus invariants, rendant l'argumentation plus réaliste et dialogique.https://www.youtube.com/watch?v=HALSBMQlSqUhttps://en.wikipedia.org/wiki/Stephen_Toulmin &lt;/p&gt; &lt;p&gt; Dans Human Understanding (1972), il propose un modèle évolutionniste du changement conceptuel en philosophie des sciences, opposé au paradigmatisme révolutionnaire de Kuhn. Les idées évoluent par innovation et sélection darwinienne, dans un &quot;champ stable&quot; partagé, évitant relativisme et absolutisme. Il défend une  &lt;a href=&quot;https://www.youtube.com/watch?v=hv7BUYzRiiU&quot;  title=&quot; le cartesian theatre de Toulmin  par Edwin gardner&quot;&gt;&quot;pluralistic conceptual relativism&quot; &lt;/a&gt;  où les concepts s'évaluent par leur pouvoir explicatif contextuel. &lt;/p&gt; &lt;p&gt; Son héritage  imprègne la rhétorique moderne, l'analyse du discours et l'éducation argumentative, favorisant des échanges constructifs intégrant réfutations. Son appel à ramener la philosophie dans la vie pratique résonne encore en éthique appliquée et en résolution de conflits. &lt;/p&gt; &#10;&#10;"/>
-    <hyperlink ref="E75" r:id="rId64" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Mary_Warnock&quot;  title=&quot; Wikipedia&quot;&gt;Mary WARNOCK&lt;/a&gt; était une  philosophe britannique spécialiste de l'éthique, de l'existentialisme et de la philosophie de l'esprit, est née Helen Mary Wilson à Winchester. Éduquée à Oxford où elle excelle en philosophie, elle devient fellow à St Hugh's College en 1949, épouse du philosophe Geoffrey Warnock, et dirige le Girton College de Cambridge (1985-1991). Élevée au rang de baronne en 1985, elle marque la sphère publique par ses rapports gouvernementaux sur l'éducation spécialisée et la fécondation in vitro. &lt;/p&gt; &lt;p&gt; Ses premiers travaux portent sur &lt;a href=&quot;https://fr.wikipedia.org/wiki/Existentialisme&quot;  title=&quot; l’existentialisme Wikipedia&quot;&gt;l'existentialisme, &lt;/a&gt;  avec des analyses de Sartre et de l'éthique existentielle dans Existentialist Ethics (1967), où elle explore la liberté et la responsabilité face à l'absurde. Dans &lt;a href=&quot;https://en.wikipedia.org/wiki/Ethics_Since_1900&quot;  title=&quot; Ethics Since 1900 Wikipedia&quot;&gt;Ethics Since 1900 &lt;/a&gt; , elle critique l'émotivisme et le préscriptivisme au profit d'une approche rationnelle et contextuelle de la morale. &lt;/p&gt; &lt;p&gt;Elle  préside deux enquêtes décisives : le rapport de 1978 intègre les enfants handicapés dans l'enseignement ordinaire via un système de &quot;statementing&quot;, qu'elle critiquera plus tard pour son coût et ses lacunes ; celui de 1984 sur l'embryologie humaine fonde la loi de 1990, régulant FIV et recherche sur embryons (limite de 14 jours), en équilibrant progrès scientifique et éthique. Défenseure d'une éthique nuancée (euthanasie assistée, intelligence animale), elle incarne une philosophie appliquée au bien commun, influençant débats sur bioéthique et éducation sans dogmatisme.&lt;/p&gt;  &#10;&#10;"/>
-    <hyperlink ref="E76" r:id="rId65" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Attila_Kot%C3%A1nyi&quot;  title=&quot; Wikipedia&quot;&gt;Attila KOTANYI&lt;/a&gt; était un poète, philosophe, écrivain et architecte-urbaniste hongrois, membre de l’Internationale situationniste entre 1960 et 1963, avant d’être exclu pour « mysticisme chrétien » et de poursuivre une pensée très originale, marquée par la critique radicale du capitalisme et par des références à la mystique juive et au bouddhisme. Il développe très tôt un marxisme non dogmatique, éloigné des partis communistes officiels, et centré sur l’idée d’un humanisme régulateur qui place l’humain créateur au centre de toutes les activités. Pour lui, &lt;a href=&quot;https://situationnisteblog.com/2022/10/31/attila-kotanyi-larchitecture-du-silence-2022/&quot;  title=&quot;attila kotanyi architecture du silence par situationniste blog&quot;&gt;l’architecture, la poésie, la peinture ou la musique &lt;/a&gt; ne sont pas des domaines séparés par leur utilité, mais des expressions d’une même activité créatrice dont le produit final est le créateur lui-même. Cette vision s’inscrit dans une volonté de dépasser la division du travail et la séparation des disciplines, en phase avec le projet marxien d’émancipation totale de l’être humain. &lt;/p&gt; &lt;p&gt; Avec Raoul Vaneigem, il cofonde le Bureau d’urbanisme unitaire, qui propose de penser l’urbanisme non comme une technique de gestion, mais comme un art des relations et de la connexion, englobant tous les autres arts. Leur « Programme élémentaire du bureau d’urbanisme unitaire » vise à créer des « espaces de ravissement » et des « châteaux situationnistes » : des environnements favorisant la rencontre, le jeu, la dérive et la construction de situations libératrices. L’idée est de transformer l’espace urbain en un terrain d’expérimentation permanente où la vie quotidienne peut devenir une œuvre collective, joyeuse et non aliénée. &lt;/p&gt; &lt;p&gt; En 1963, il est exclu de &lt;a href=&quot;https://www.youtube.com/watch?v=2IaFG-HWBms&quot;  title=&quot;150ans de la commune thèse situationniste par libradio genève&quot;&gt;l’Internationale situationniste &lt;/a&gt; pour son « mysticisme chrétien », car il défend la thèse de l’impossibilité d’un art non corrompu et s’intéresse aux traditions mystiques, notamment chrétiennes, mais aussi juives et bouddhistes. Dans les années 1990, de retour à Budapest, il anime un cercle de jeunes intellectuels lors de rencontres hebdomadaires où il élabore sa théorie du Shabbat, conçue comme une suspension radicale de l’activité productive et un temps de résistance au capitalisme. Cette « théorie du Shabbat » prolonge sa critique de la société du spectacle en proposant un temps sacré, non marchand, où l’être humain peut échapper à la logique du travail et de la performance. &lt;/p&gt; &lt;p&gt; Sa  philosophie de se caractérise par une radicalité fondée sur la subjectivité, nourrie aussi bien par le marxisme que par la mystique juive, le bouddhisme et diverses traditions spirituelles. Sa pensée articule critique sociale et quête existentielle : il ne s’agit pas seulement de transformer les structures économiques et urbaines, mais aussi de libérer la vie intérieure, la créativité et la capacité de jouir sans entraves. En ce sens, il apparaît comme un penseur de la résistance intérieure et de la création d’espaces (concrets et symboliques) où l’humain peut redevenir sujet de sa propre existence. &lt;/p&gt; &#10;&#10;"/>
-    <hyperlink ref="H76" r:id="rId66" display="https://www.laphilo.fr/pho/akotanyi-mini.webp"/>
-    <hyperlink ref="I76" r:id="rId67" display="https://www.laphilo.fr/photo/akotanyi.webp"/>
-    <hyperlink ref="E77" r:id="rId68" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Anthony_Quinton&quot;  title=&quot; Wikipedia&quot;&gt;Anthony QUINTON&lt;/a&gt;  était un philosophe politique et moral anglais, métaphysicien et matérialiste, est une figure oxonienne conservatrice. Éduqué à Christ Church (Oxford) après un service dans la RAF, il fut Fellow à All Souls (1949-1955), tutor à New College, puis président de Trinity College (1978-1987). Pair à vie (Baron Quinton) depuis 1983, il présida la British Library (1985-1990) et anima Round Britain Quiz à la BBC. &lt;/p&gt; &lt;p&gt; Dans The Politics of Imperfection (1978), il théorise le conservatisme britannique comme marqué par le traditionalisme (valeur de ce qui résiste au temps), l'organicisme (société comme organisme historique) et le scepticisme politique (méfiance envers les utopies rationnelles). Inspiré par &lt;a href=&quot;https://www.persee.fr/doc/dhs_0070-6760_2001_num_33_1_2448_t1_0691_0000_3&quot;  title=&quot; Anthony Quinton Hume 2000  par Persée&quot;&gt;Hume et Hooker, &lt;/a&gt;  il oppose cette sagesse collective empirique aux idéaux abstraits de la gauche, prônant une évolution prudente des institutions.https://www.youtube.com/watch?v=-qV2YFhKES8https://www.reddit.com/r/PoliticalPhilosophy/comments/15vj8do/foundational_texts_on_conservativism/ &lt;/p&gt; &lt;p&gt; En métaphysique, il défend un  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Nominalisme&quot;  title=&quot; nominalisme par Wikipedia&quot;&gt;nominalisme &lt;/a&gt; des classes naturelles : les propriétés sont des classes objectives de choses similaires, évitant le réalisme des universaux sans tomber dans le subjectivisme pur. Matérialiste de l'esprit, il analyse la conscience comme fonction du cerveau, tout en valorisant le sens commun contre les excès analytiques ou continentaux. &lt;/p&gt; &lt;p&gt; Auteur prolifique (ouvrages sur Hume, The Nature of Things), admirateur de Thatcher, il incarne un  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Conservatisme&quot;  title=&quot; conservatisme par Wikipedia&quot;&gt;conservatisme &lt;/a&gt; intellectuel élégant, influençant la philosophie morale et politique par son réalisme sceptique. Son legs persiste dans les débats sur tradition et rationalité politique. &lt;/p&gt; &#10;&#10;"/>
-    <hyperlink ref="H77" r:id="rId69" display="https://www.laphilo.fr/pho/quinton-mini.webp"/>
-    <hyperlink ref="I77" r:id="rId70" display="https://laphilo.fr/photo/akotanyi.webp"/>
-    <hyperlink ref="H80" r:id="rId71" display="https://www.laphilo.fr/pho/sbeer-mini.webp"/>
-    <hyperlink ref="E82" r:id="rId72" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Geoffrey_Warnock&quot;  title=&quot; Wikipedia&quot;&gt;Geoffrey WARNOCK&lt;/a&gt;  était un philosophe anglais de l’ordinaire, formé à Oxford après un service militaire dans les Irish Guards. Fellow à Magdalen College dès 1949, puis Principal de Hertford College (1971-1988) et Vice-Chancelier d’Oxford (1981-1985), il est connu pour avoir édité et publié les œuvres posthumes de J.L. Austin, dont Philosophical Papers et Sense and Sensibilia. &lt;/p&gt; &lt;p&gt; Dans Contemporary Moral Philosophy (1967), il critique l’émotivisme et le préscriptivisme (Ayer, Stevenson, Hare) pour leur réduction du discours moral à des attitudes ou impératifs sans justification rationnelle. Il prône un retour à un &lt;a href=&quot;https://fr.wikipedia.org/wiki/Intuitionnisme_social&quot;   title=&quot;L’intuitionnisme par Kikipedia&quot;&gt;intuitionnisme réformé, &lt;/a&gt;  où les jugements moraux s’appuient sur des considérations objectives et partagées, comme le bien-être humain, sans dogmatisme. &lt;/p&gt; &lt;p&gt; Il  défend une éthique pratique et modérée, opposée aux excès relativistes ou formalistes, valorisant le rôle du philosophe dans l’analyse claire des concepts moraux ordinaires. Proche de son épouse Mary Warnock (philosophe éthicienne), il incarne l’Oxford analytique appliquée à la vie publique. &lt;/p&gt; &lt;p&gt; Son legs, discret mais solide, influence la philosophie morale britannique par son équilibre entre rigueur logique et humanisme concret, reliant Austin et Williams dans une tradition oxonienne sceptique. &lt;/p&gt; "/>
-    <hyperlink ref="E84" r:id="rId73" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Pierre_Hassner&quot;  title=&quot; Wikipedia&quot;&gt;Pierre HASNER&lt;/a&gt; était un philosophe politique français d’origine roumaine, figure de la pensée européenne sur la guerre, le totalitarisme et la politique mondiale. Formé à la philosophie (École normale supérieure, agrégation en 1952) et proche de Raymond Aron, il a fait de la philosophie le socle de son analyse des relations internationales, cherchant à éclairer les problèmes géopolitiques par la pensée politique et morale. &lt;/p&gt; &lt;p&gt; Il se distingue par une approche qui combine philosophie politique et sociologie historique des relations internationales. Il est considéré comme inclassable, étant décrit comme « réaliste » (car il prend toujours en compte les contraintes du politique), « libéral » (car il insiste sur les normes et les droits de l’homme) et même « constructiviste » (par son intérêt pour le rôle des idées dans les RI). Sa pensée a marqué l’étude de la guerre froide, puis  &lt;a href=&quot;https://lediplomate.media/portrait-pierre-hassner-philosophe-interprete-inclassable-monde-desordonne/&quot;  title=&quot;pierre hassner philosophe fracture d’un monde desordonné par lediplomate&quot;&gt;celle des conflits de l’après-guerre &lt;/a&gt;  froide, notamment terrorisme, guerres hybrides et « nettoyage ethnique ». &lt;/p&gt; &lt;p&gt; Parmi ses œuvres majeures, on trouve La Violence et la Paix, La Terreur et l’Empire (2003), Washington et le Monde. Dilemmes d’une superpuissance (2003, avec Justin Vaïsse) et La Revanche des passions. Métamorphoses de la violence et crises du politique (2015). Il développe une réflexion sur la géopolitique des passions, soulignant que la guerre n’est pas un état « clair et distinct », mais une réalité diffuse et graduelle, marquée par les conflits hybrides, le terrorisme islamiste et la montée des violences politiques et identitaires. Pour lui, le totalitarisme et la guerre sont deux fléaux qu’il tente de comprendre pour essayer de surmonter leurs causes. &lt;/p&gt; &lt;p&gt; Il est souvent présenté comme un disciple de Raymond Aron, reprenant sa tradition de philosophie politique appliquée aux grandes questions internationales : guerre, paix, puissance, valeurs. Il n’est pas rattaché à un courant strict (réaliste, libéral, constructiviste) mais incarne une  &lt;a href=&quot;https://www.youtube.com/watch?v=9XnlKLbbm2Q&quot;  title=&quot;pierre hassner par smolar web of stories&quot;&gt;forme de pensée politique &lt;/a&gt; ouverte, qui refuse les catégories rigides et cherche à comprendre la complexité du monde à partir de la philosophie. Il reste une référence incontournable pour ceux qui veulent penser la guerre, la paix et la politique mondiale sans se limiter à des schémas académiques fermés, et son héritage est considéré comme plus urgent que jamais dans un monde marqué par les crises géopolitiques contemporaines. &lt;/p&gt; &#10; &lt;audio controls title=&quot;pierre Hassner par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/11189-26.11.2015-ITEMA_20849989-2015C15000E0181-ITE_00077318_RSCE-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; &#10;&#10;"/>
-    <hyperlink ref="H85" r:id="rId74" display="https://www.laphilo.fr/pho/lluisifont-mini.webp"/>
-    <hyperlink ref="E87" r:id="rId75" display="&lt;p&gt;&lt;a href=&quot;https://es.wikipedia.org/wiki/Javier_Muguerza&quot;   title=&quot; Wikipedia&quot;&gt;Javier MURGUERZA&lt;/a&gt;  était un philosophe espagnol majeur, disciple de José Luis López Aranguren et José Ferrater Mora, connu pour son &lt;a href=&quot;https://fr.wikipedia.org/wiki/Agnosticisme&quot;  title=&quot; Agnosticisme  par Wikipedia&quot;&gt;l'agnosticisme &lt;/a&gt; déclaré et sa défense de la &quot;perplexité&quot; comme posture éthique et rationnelle face aux certitudes dogmatiques. Né à Coín (Malaga), il a doctoré en 1965 à l'Université Complutense de Madrid avec une thèse sur Frege, avant de devenir catedrático en philosophie morale dans plusieurs universités (La Laguna, Autónoma de Barcelona, UNED). Il a fondé l'Institut de Philosophie du CSIC et la revue Isegoría en 1990, promouvant un dialogue ibéro-américain en philosophie morale et politique. &lt;/p&gt; &lt;p&gt; Bien que non lié à l'origine historique de l'agnosticisme (Huxley, 1869), Muguerza en incarne une version moderne et personnelle, influencée par Kant et la philosophie critique. Dans des essais comme « La profession de foi de l'incroyant », il adopte une position agnostique : vivre « comme si Dieu n'existait pas » tout en reconnaissant que la solidarité humaine pourrait requérir une motivation quasi-religieuse pour transcender la simple justice. Sa pensée, marquée par La raison sans espoir (1977) et Depuis la perplexité (1990), valorise le dissensus et l'impératif de la dissidence contre tout autoritarisme, y compris religieux. &lt;/p&gt; &lt;p&gt; Il dialogue ouvertement avec la théologie chrétienne tout en maintenant une laïcité ferme, analysant des dilemmes comme la question socratique d'Euthyphron (Dieu fonde-t-il la morale ?) ou le problème du mal d'Épicure. Il critique les éthiques religieuses pour leur risque de subordonner la morale à la religion, plaidant pour une éthique publique cosmopolite et utopique, sans recours à une loi naturelle théologique. Ses &quot;trois Critiques&quot; (analytique, dialogique, onirique) renouvellent Kant en soulignant l'incertitude rationnelle. &lt;/p&gt; &lt;p&gt; Figure de la transition démocratique espagnole, il a dirigé plus de vingt thèses et reçu un doctorat honoris causa de La Laguna en 2007. Son legs : une philosophie du dissensus qui fait écho à l'agnosticisme en refusant les réponses absolues, favorisant une raison perpleja et engagée. &lt;/p&gt; &#10;"/>
-    <hyperlink ref="H87" r:id="rId76" display="https://laphilo.fr/pho/jmuguerza-mini.webp"/>
-    <hyperlink ref="H88" r:id="rId77" display="https://www.laphilo.fr/pho/parfit-mini.webp"/>
-    <hyperlink ref="E89" r:id="rId78" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/L%C3%A1szl%C3%B3_Tengelyi&quot;   title=&quot; Wikipedia&quot;&gt;Laszlo TENGELYI&lt;/a&gt;  était un philosophe hongrois renommé, spécialiste de phénoménologie, qui n'est pas directement associé à l'agnosticisme dans ses travaux principaux, mais dont la réflexion philosophique touche aux limites de la connaissance humaine, un thème proche. Né à Budapest, il a étudié à l'université Eötvös Loránd avant de poursuivre une carrière académique en Allemagne, notamment comme professeur à l'université de Wuppertal à partir de 2001, succédant à Klaus Held sur la chaire de phénoménologie et philosophie théorétique. &lt;/p&gt; &lt;p&gt; Ses recherches se concentraient sur la phénoménologie husserlienne, le kantisme et la &quot;nouvelle phénoménologie&quot; française, comme chez Levinas ou Marion, explorant l'expérience de la singularité, l'affectivité et les rapports entre monde fini et infini. Dans des ouvrages tels que Neue Phänomenologie in Frankreich (2012) ou Welt und Unendlichkeit (posthume, 2014), il questionne les fondements de la métaphysique  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Ph%C3%A9nom%C3%A9nologie_(philosophie)&quot;  title=&quot; Phénoménologie  par Wikipedia&quot;&gt;phénoménologique, &lt;/a&gt; sans aborder explicitement l'agnosticisme, mais en soulignant les horizons inconnaissables de l'expérience. &lt;/p&gt; &lt;p&gt; Bien qu'aucun lien direct n'apparaisse avec l'origine de  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Agnosticisme&quot;  title=&quot; Agnosticisme  par Wikipedia&quot;&gt;l'agnosticisme &lt;/a&gt;  – forgé par Thomas Huxley en 1869 et remontant à Protagoras –, Tengelyi a contribué à des débats sur la connaissance et l'absolu via son engagement dans des revues comme Annales de phénoménologie. Un document mentionne &quot;di-agnostique Henry&quot; près de son nom, peut-être une référence contextuelle à des discussions philosophiques sur le doute épistémologique, mais cela reste marginal. &lt;/p&gt; &lt;p&gt; Il i reste une figure clé de la phénoménologie contemporaine européenne, avec des publications en hongrois, allemand et français, et un engagement public, comme sa lettre ouverte en 2011 défendant des intellectuels hongrois face à des attaques médiatiques. &lt;/p&gt; &#10;&#10;"/>
-    <hyperlink ref="H89" r:id="rId79" display="https://laphilo.fr/pho/ltengelyi-mini.webp"/>
+    <hyperlink ref="E67" r:id="rId60" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Alfred_Jules_Ayer&quot; title=&quot; Wikipedia&quot;&gt;Alfred Jules AYER&lt;/a&gt; souvent surnommé « Freddie », était un philosophe britannique qui a joué un rôle central dans la diffusion du positivisme logique dans le monde anglophone. Né à Londres dans une famille d’origine suisse et néerlandaise, il fait ses études à Eton puis à Oxford, où il devient rapidement  &lt;a href=&quot;https://www.la-philosophie.fr/philosophie-analytique/alfred-jules-ayer-8.html&quot;  title=&quot;philosophie analytique par la philosophie&quot;&gt; une figure majeure &lt;/a&gt; de la philosophie analytique. C’est à seulement 24 ans qu’il publie son ouvrage le plus célèbre, Language, Truth, and Logic (1936), qui expose avec clarté et rigueur les thèses fondamentales du Cercle de Vienne et établit sa réputation internationale. &lt;/p&gt; &lt;p&gt; Au cœur de sa philosophie se trouve le principe de vérification, selon lequel une proposition n’a de sens cognitif que si elle est soit analytique (vraie en vertu de la signification des termes, comme en logique ou en mathématiques), soit empiriquement vérifiable (c’est-à-dire susceptible d’être confirmée ou infirmée par l’expérience). Ce critère lui permet de rejeter comme dénuées de sens littéral la plupart des affirmations de la métaphysique traditionnelle, de la théologie spéculative et de certaines formes d’éthique normative : elles ne sont pas fausses, mais simplement non vérifiables, donc dépourvues de contenu factuel. Il distingue ainsi strictement la philosophie, conçue comme analyse logique du langage, des sciences empiriques, seules habilitées à produire des connaissances sur le monde. &lt;/p&gt; &lt;p&gt; En éthique, il défend une position connue sous  &lt;a href=&quot;https://www.youtube.com/watch?v=HG5kIR6iF8g&quot;  title=&quot;A,J, Ayer’s Emotivism par philosophy Vibe&quot;&gt;le nom d’émotivisme. &lt;/a&gt;  Selon lui, les jugements moraux (« Le vol est mal », « La générosité est bonne ») n’expriment pas des faits objectifs, car il n’existe pas de « faits moraux » vérifiables empiriquement. Ils sont plutôt l’expression d’attitudes émotionnelles ou de prescriptions destinées à influencer les comportements d’autrui. Cette thèse s’inscrit dans une distinction radicale entre faits et valeurs : la science et la logique peuvent traiter des premiers, mais les secondes relèvent de la subjectivité et ne peuvent fonder aucune connaissance objective. &lt;/p&gt; &lt;p&gt; Au fil de sa carrière, il a nuancé certaines de ses positions initiales, notamment en reformulant le principe de vérification pour répondre aux objections (par exemple, en distinguant vérification directe et indirecte). Il a aussi évolué sur des questions de perception, de causalité et de liberté, tout en restant fidèle à un empirisme rigoureux et à une méfiance envers toute forme de métaphysique spéculative. Malgré les critiques ultérieures adressées au positivisme logique — notamment sur le statut même du principe de vérification —, son influence sur la philosophie analytique du XXᵉ siècle reste profonde, en particulier dans les débats sur le sens, la connaissance et l’éthique. &lt;/p&gt; &#10;&#10;&#10;"/>
+    <hyperlink ref="H67" r:id="rId61" display="https://www.laphilo.fr/pho/ajayer-mini.webp"/>
+    <hyperlink ref="H68" r:id="rId62" display="https://www.laphilo.fr/pho/jlaustin-mini.webp"/>
+    <hyperlink ref="H70" r:id="rId63" display="https://www.laphilo.fr/pho/pgrice-mini.webp"/>
+    <hyperlink ref="H72" r:id="rId64" display="https://www.laphilo.fr/pho/eanscombe-mini.webp"/>
+    <hyperlink ref="E74" r:id="rId65" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Stephen_Toulmin&quot;  title=&quot; Wikipedia&quot;&gt;Stephen TOULMIN&lt;/a&gt;  était un philosophe britanique  influencé par Wittgenstein, est un penseur majeur de la philosophie des sciences et de l'argumentation pratique. Né en Angleterre, il étudie à Cambridge, enseigne à Oxford, Leeds, puis aux États-Unis (notamment à Northwestern et USC). Critique du formalisme logique absolu, il prône une approche contextualisée des raisonnements, applicable au droit, à la médecine ou à la diplomatie, loin des abstractions syllogistiques. &lt;/p&gt; &lt;p&gt; Son œuvre fondatrice, The Uses of Argument (1958), introduit le  &lt;a href=&quot;https://www.youtube.com/watch?v=J1WDW2F-KBs&quot;  title=&quot; le modèle de Toulmin  par Mooc Cyu&quot;&gt;modèle d'argumentation de Toulmin &lt;/a&gt;  : une structure à six composantes pour analyser les débats réels. La claim (thèse), les grounds (données), le warrant (justification liant données et thèse), le backing (soutien du warrant), les qualifiers (modalisateurs comme &quot;probablement&quot;), et les rebuttals (contre-arguments). Ce schéma met en lumière les aspects &quot;field-dependent&quot; (dépendants du domaine) versus invariants, rendant l'argumentation plus réaliste et dialogique.https://www.youtube.com/watch?v=HALSBMQlSqUhttps://en.wikipedia.org/wiki/Stephen_Toulmin &lt;/p&gt; &lt;p&gt; Dans Human Understanding (1972), il propose un modèle évolutionniste du changement conceptuel en philosophie des sciences, opposé au paradigmatisme révolutionnaire de Kuhn. Les idées évoluent par innovation et sélection darwinienne, dans un &quot;champ stable&quot; partagé, évitant relativisme et absolutisme. Il défend une  &lt;a href=&quot;https://www.youtube.com/watch?v=hv7BUYzRiiU&quot;  title=&quot; le cartesian theatre de Toulmin  par Edwin gardner&quot;&gt;&quot;pluralistic conceptual relativism&quot; &lt;/a&gt;  où les concepts s'évaluent par leur pouvoir explicatif contextuel. &lt;/p&gt; &lt;p&gt; Son héritage  imprègne la rhétorique moderne, l'analyse du discours et l'éducation argumentative, favorisant des échanges constructifs intégrant réfutations. Son appel à ramener la philosophie dans la vie pratique résonne encore en éthique appliquée et en résolution de conflits. &lt;/p&gt; &#10;&#10;"/>
+    <hyperlink ref="E76" r:id="rId66" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Mary_Warnock&quot;  title=&quot; Wikipedia&quot;&gt;Mary WARNOCK&lt;/a&gt; était une  philosophe britannique spécialiste de l'éthique, de l'existentialisme et de la philosophie de l'esprit, est née Helen Mary Wilson à Winchester. Éduquée à Oxford où elle excelle en philosophie, elle devient fellow à St Hugh's College en 1949, épouse du philosophe Geoffrey Warnock, et dirige le Girton College de Cambridge (1985-1991). Élevée au rang de baronne en 1985, elle marque la sphère publique par ses rapports gouvernementaux sur l'éducation spécialisée et la fécondation in vitro. &lt;/p&gt; &lt;p&gt; Ses premiers travaux portent sur &lt;a href=&quot;https://fr.wikipedia.org/wiki/Existentialisme&quot;  title=&quot; l’existentialisme Wikipedia&quot;&gt;l'existentialisme, &lt;/a&gt;  avec des analyses de Sartre et de l'éthique existentielle dans Existentialist Ethics (1967), où elle explore la liberté et la responsabilité face à l'absurde. Dans &lt;a href=&quot;https://en.wikipedia.org/wiki/Ethics_Since_1900&quot;  title=&quot; Ethics Since 1900 Wikipedia&quot;&gt;Ethics Since 1900 &lt;/a&gt; , elle critique l'émotivisme et le préscriptivisme au profit d'une approche rationnelle et contextuelle de la morale. &lt;/p&gt; &lt;p&gt;Elle  préside deux enquêtes décisives : le rapport de 1978 intègre les enfants handicapés dans l'enseignement ordinaire via un système de &quot;statementing&quot;, qu'elle critiquera plus tard pour son coût et ses lacunes ; celui de 1984 sur l'embryologie humaine fonde la loi de 1990, régulant FIV et recherche sur embryons (limite de 14 jours), en équilibrant progrès scientifique et éthique. Défenseure d'une éthique nuancée (euthanasie assistée, intelligence animale), elle incarne une philosophie appliquée au bien commun, influençant débats sur bioéthique et éducation sans dogmatisme.&lt;/p&gt;  &#10;&#10;"/>
+    <hyperlink ref="E77" r:id="rId67" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Attila_Kot%C3%A1nyi&quot;  title=&quot; Wikipedia&quot;&gt;Attila KOTANYI&lt;/a&gt; était un poète, philosophe, écrivain et architecte-urbaniste hongrois, membre de l’Internationale situationniste entre 1960 et 1963, avant d’être exclu pour « mysticisme chrétien » et de poursuivre une pensée très originale, marquée par la critique radicale du capitalisme et par des références à la mystique juive et au bouddhisme. Il développe très tôt un marxisme non dogmatique, éloigné des partis communistes officiels, et centré sur l’idée d’un humanisme régulateur qui place l’humain créateur au centre de toutes les activités. Pour lui, &lt;a href=&quot;https://situationnisteblog.com/2022/10/31/attila-kotanyi-larchitecture-du-silence-2022/&quot;  title=&quot;attila kotanyi architecture du silence par situationniste blog&quot;&gt;l’architecture, la poésie, la peinture ou la musique &lt;/a&gt; ne sont pas des domaines séparés par leur utilité, mais des expressions d’une même activité créatrice dont le produit final est le créateur lui-même. Cette vision s’inscrit dans une volonté de dépasser la division du travail et la séparation des disciplines, en phase avec le projet marxien d’émancipation totale de l’être humain. &lt;/p&gt; &lt;p&gt; Avec Raoul Vaneigem, il cofonde le Bureau d’urbanisme unitaire, qui propose de penser l’urbanisme non comme une technique de gestion, mais comme un art des relations et de la connexion, englobant tous les autres arts. Leur « Programme élémentaire du bureau d’urbanisme unitaire » vise à créer des « espaces de ravissement » et des « châteaux situationnistes » : des environnements favorisant la rencontre, le jeu, la dérive et la construction de situations libératrices. L’idée est de transformer l’espace urbain en un terrain d’expérimentation permanente où la vie quotidienne peut devenir une œuvre collective, joyeuse et non aliénée. &lt;/p&gt; &lt;p&gt; En 1963, il est exclu de &lt;a href=&quot;https://www.youtube.com/watch?v=2IaFG-HWBms&quot;  title=&quot;150ans de la commune thèse situationniste par libradio genève&quot;&gt;l’Internationale situationniste &lt;/a&gt; pour son « mysticisme chrétien », car il défend la thèse de l’impossibilité d’un art non corrompu et s’intéresse aux traditions mystiques, notamment chrétiennes, mais aussi juives et bouddhistes. Dans les années 1990, de retour à Budapest, il anime un cercle de jeunes intellectuels lors de rencontres hebdomadaires où il élabore sa théorie du Shabbat, conçue comme une suspension radicale de l’activité productive et un temps de résistance au capitalisme. Cette « théorie du Shabbat » prolonge sa critique de la société du spectacle en proposant un temps sacré, non marchand, où l’être humain peut échapper à la logique du travail et de la performance. &lt;/p&gt; &lt;p&gt; Sa  philosophie de se caractérise par une radicalité fondée sur la subjectivité, nourrie aussi bien par le marxisme que par la mystique juive, le bouddhisme et diverses traditions spirituelles. Sa pensée articule critique sociale et quête existentielle : il ne s’agit pas seulement de transformer les structures économiques et urbaines, mais aussi de libérer la vie intérieure, la créativité et la capacité de jouir sans entraves. En ce sens, il apparaît comme un penseur de la résistance intérieure et de la création d’espaces (concrets et symboliques) où l’humain peut redevenir sujet de sa propre existence. &lt;/p&gt; &#10;&#10;"/>
+    <hyperlink ref="H77" r:id="rId68" display="https://www.laphilo.fr/pho/akotanyi-mini.webp"/>
+    <hyperlink ref="I77" r:id="rId69" display="https://www.laphilo.fr/photo/akotanyi.webp"/>
+    <hyperlink ref="E78" r:id="rId70" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Anthony_Quinton&quot;  title=&quot; Wikipedia&quot;&gt;Anthony QUINTON&lt;/a&gt;  était un philosophe politique et moral anglais, métaphysicien et matérialiste, est une figure oxonienne conservatrice. Éduqué à Christ Church (Oxford) après un service dans la RAF, il fut Fellow à All Souls (1949-1955), tutor à New College, puis président de Trinity College (1978-1987). Pair à vie (Baron Quinton) depuis 1983, il présida la British Library (1985-1990) et anima Round Britain Quiz à la BBC. &lt;/p&gt; &lt;p&gt; Dans The Politics of Imperfection (1978), il théorise le conservatisme britannique comme marqué par le traditionalisme (valeur de ce qui résiste au temps), l'organicisme (société comme organisme historique) et le scepticisme politique (méfiance envers les utopies rationnelles). Inspiré par &lt;a href=&quot;https://www.persee.fr/doc/dhs_0070-6760_2001_num_33_1_2448_t1_0691_0000_3&quot;  title=&quot; Anthony Quinton Hume 2000  par Persée&quot;&gt;Hume et Hooker, &lt;/a&gt;  il oppose cette sagesse collective empirique aux idéaux abstraits de la gauche, prônant une évolution prudente des institutions.https://www.youtube.com/watch?v=-qV2YFhKES8https://www.reddit.com/r/PoliticalPhilosophy/comments/15vj8do/foundational_texts_on_conservativism/ &lt;/p&gt; &lt;p&gt; En métaphysique, il défend un  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Nominalisme&quot;  title=&quot; nominalisme par Wikipedia&quot;&gt;nominalisme &lt;/a&gt; des classes naturelles : les propriétés sont des classes objectives de choses similaires, évitant le réalisme des universaux sans tomber dans le subjectivisme pur. Matérialiste de l'esprit, il analyse la conscience comme fonction du cerveau, tout en valorisant le sens commun contre les excès analytiques ou continentaux. &lt;/p&gt; &lt;p&gt; Auteur prolifique (ouvrages sur Hume, The Nature of Things), admirateur de Thatcher, il incarne un  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Conservatisme&quot;  title=&quot; conservatisme par Wikipedia&quot;&gt;conservatisme &lt;/a&gt; intellectuel élégant, influençant la philosophie morale et politique par son réalisme sceptique. Son legs persiste dans les débats sur tradition et rationalité politique. &lt;/p&gt; &#10;&#10;"/>
+    <hyperlink ref="H78" r:id="rId71" display="https://www.laphilo.fr/pho/quinton-mini.webp"/>
+    <hyperlink ref="I78" r:id="rId72" display="https://laphilo.fr/photo/akotanyi.webp"/>
+    <hyperlink ref="H81" r:id="rId73" display="https://www.laphilo.fr/pho/sbeer-mini.webp"/>
+    <hyperlink ref="E83" r:id="rId74" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Geoffrey_Warnock&quot;  title=&quot; Wikipedia&quot;&gt;Geoffrey WARNOCK&lt;/a&gt;  était un philosophe anglais de l’ordinaire, formé à Oxford après un service militaire dans les Irish Guards. Fellow à Magdalen College dès 1949, puis Principal de Hertford College (1971-1988) et Vice-Chancelier d’Oxford (1981-1985), il est connu pour avoir édité et publié les œuvres posthumes de J.L. Austin, dont Philosophical Papers et Sense and Sensibilia. &lt;/p&gt; &lt;p&gt; Dans Contemporary Moral Philosophy (1967), il critique l’émotivisme et le préscriptivisme (Ayer, Stevenson, Hare) pour leur réduction du discours moral à des attitudes ou impératifs sans justification rationnelle. Il prône un retour à un &lt;a href=&quot;https://fr.wikipedia.org/wiki/Intuitionnisme_social&quot;   title=&quot;L’intuitionnisme par Kikipedia&quot;&gt;intuitionnisme réformé, &lt;/a&gt;  où les jugements moraux s’appuient sur des considérations objectives et partagées, comme le bien-être humain, sans dogmatisme. &lt;/p&gt; &lt;p&gt; Il  défend une éthique pratique et modérée, opposée aux excès relativistes ou formalistes, valorisant le rôle du philosophe dans l’analyse claire des concepts moraux ordinaires. Proche de son épouse Mary Warnock (philosophe éthicienne), il incarne l’Oxford analytique appliquée à la vie publique. &lt;/p&gt; &lt;p&gt; Son legs, discret mais solide, influence la philosophie morale britannique par son équilibre entre rigueur logique et humanisme concret, reliant Austin et Williams dans une tradition oxonienne sceptique. &lt;/p&gt; "/>
+    <hyperlink ref="E85" r:id="rId75" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Pierre_Hassner&quot;  title=&quot; Wikipedia&quot;&gt;Pierre HASNER&lt;/a&gt; était un philosophe politique français d’origine roumaine, figure de la pensée européenne sur la guerre, le totalitarisme et la politique mondiale. Formé à la philosophie (École normale supérieure, agrégation en 1952) et proche de Raymond Aron, il a fait de la philosophie le socle de son analyse des relations internationales, cherchant à éclairer les problèmes géopolitiques par la pensée politique et morale. &lt;/p&gt; &lt;p&gt; Il se distingue par une approche qui combine philosophie politique et sociologie historique des relations internationales. Il est considéré comme inclassable, étant décrit comme « réaliste » (car il prend toujours en compte les contraintes du politique), « libéral » (car il insiste sur les normes et les droits de l’homme) et même « constructiviste » (par son intérêt pour le rôle des idées dans les RI). Sa pensée a marqué l’étude de la guerre froide, puis  &lt;a href=&quot;https://lediplomate.media/portrait-pierre-hassner-philosophe-interprete-inclassable-monde-desordonne/&quot;  title=&quot;pierre hassner philosophe fracture d’un monde desordonné par lediplomate&quot;&gt;celle des conflits de l’après-guerre &lt;/a&gt;  froide, notamment terrorisme, guerres hybrides et « nettoyage ethnique ». &lt;/p&gt; &lt;p&gt; Parmi ses œuvres majeures, on trouve La Violence et la Paix, La Terreur et l’Empire (2003), Washington et le Monde. Dilemmes d’une superpuissance (2003, avec Justin Vaïsse) et La Revanche des passions. Métamorphoses de la violence et crises du politique (2015). Il développe une réflexion sur la géopolitique des passions, soulignant que la guerre n’est pas un état « clair et distinct », mais une réalité diffuse et graduelle, marquée par les conflits hybrides, le terrorisme islamiste et la montée des violences politiques et identitaires. Pour lui, le totalitarisme et la guerre sont deux fléaux qu’il tente de comprendre pour essayer de surmonter leurs causes. &lt;/p&gt; &lt;p&gt; Il est souvent présenté comme un disciple de Raymond Aron, reprenant sa tradition de philosophie politique appliquée aux grandes questions internationales : guerre, paix, puissance, valeurs. Il n’est pas rattaché à un courant strict (réaliste, libéral, constructiviste) mais incarne une  &lt;a href=&quot;https://www.youtube.com/watch?v=9XnlKLbbm2Q&quot;  title=&quot;pierre hassner par smolar web of stories&quot;&gt;forme de pensée politique &lt;/a&gt; ouverte, qui refuse les catégories rigides et cherche à comprendre la complexité du monde à partir de la philosophie. Il reste une référence incontournable pour ceux qui veulent penser la guerre, la paix et la politique mondiale sans se limiter à des schémas académiques fermés, et son héritage est considéré comme plus urgent que jamais dans un monde marqué par les crises géopolitiques contemporaines. &lt;/p&gt; &#10; &lt;audio controls title=&quot;pierre Hassner par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/11189-26.11.2015-ITEMA_20849989-2015C15000E0181-ITE_00077318_RSCE-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; &#10;&#10;"/>
+    <hyperlink ref="H86" r:id="rId76" display="https://www.laphilo.fr/pho/lluisifont-mini.webp"/>
+    <hyperlink ref="E88" r:id="rId77" display="&lt;p&gt;&lt;a href=&quot;https://es.wikipedia.org/wiki/Javier_Muguerza&quot;   title=&quot; Wikipedia&quot;&gt;Javier MURGUERZA&lt;/a&gt;  était un philosophe espagnol majeur, disciple de José Luis López Aranguren et José Ferrater Mora, connu pour son &lt;a href=&quot;https://fr.wikipedia.org/wiki/Agnosticisme&quot;  title=&quot; Agnosticisme  par Wikipedia&quot;&gt;l'agnosticisme &lt;/a&gt; déclaré et sa défense de la &quot;perplexité&quot; comme posture éthique et rationnelle face aux certitudes dogmatiques. Né à Coín (Malaga), il a doctoré en 1965 à l'Université Complutense de Madrid avec une thèse sur Frege, avant de devenir catedrático en philosophie morale dans plusieurs universités (La Laguna, Autónoma de Barcelona, UNED). Il a fondé l'Institut de Philosophie du CSIC et la revue Isegoría en 1990, promouvant un dialogue ibéro-américain en philosophie morale et politique. &lt;/p&gt; &lt;p&gt; Bien que non lié à l'origine historique de l'agnosticisme (Huxley, 1869), Muguerza en incarne une version moderne et personnelle, influencée par Kant et la philosophie critique. Dans des essais comme « La profession de foi de l'incroyant », il adopte une position agnostique : vivre « comme si Dieu n'existait pas » tout en reconnaissant que la solidarité humaine pourrait requérir une motivation quasi-religieuse pour transcender la simple justice. Sa pensée, marquée par La raison sans espoir (1977) et Depuis la perplexité (1990), valorise le dissensus et l'impératif de la dissidence contre tout autoritarisme, y compris religieux. &lt;/p&gt; &lt;p&gt; Il dialogue ouvertement avec la théologie chrétienne tout en maintenant une laïcité ferme, analysant des dilemmes comme la question socratique d'Euthyphron (Dieu fonde-t-il la morale ?) ou le problème du mal d'Épicure. Il critique les éthiques religieuses pour leur risque de subordonner la morale à la religion, plaidant pour une éthique publique cosmopolite et utopique, sans recours à une loi naturelle théologique. Ses &quot;trois Critiques&quot; (analytique, dialogique, onirique) renouvellent Kant en soulignant l'incertitude rationnelle. &lt;/p&gt; &lt;p&gt; Figure de la transition démocratique espagnole, il a dirigé plus de vingt thèses et reçu un doctorat honoris causa de La Laguna en 2007. Son legs : une philosophie du dissensus qui fait écho à l'agnosticisme en refusant les réponses absolues, favorisant une raison perpleja et engagée. &lt;/p&gt; &#10;"/>
+    <hyperlink ref="H88" r:id="rId78" display="https://laphilo.fr/pho/jmuguerza-mini.webp"/>
+    <hyperlink ref="H89" r:id="rId79" display="https://www.laphilo.fr/pho/parfit-mini.webp"/>
+    <hyperlink ref="E90" r:id="rId80" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/L%C3%A1szl%C3%B3_Tengelyi&quot;   title=&quot; Wikipedia&quot;&gt;Laszlo TENGELYI&lt;/a&gt;  était un philosophe hongrois renommé, spécialiste de phénoménologie, qui n'est pas directement associé à l'agnosticisme dans ses travaux principaux, mais dont la réflexion philosophique touche aux limites de la connaissance humaine, un thème proche. Né à Budapest, il a étudié à l'université Eötvös Loránd avant de poursuivre une carrière académique en Allemagne, notamment comme professeur à l'université de Wuppertal à partir de 2001, succédant à Klaus Held sur la chaire de phénoménologie et philosophie théorétique. &lt;/p&gt; &lt;p&gt; Ses recherches se concentraient sur la phénoménologie husserlienne, le kantisme et la &quot;nouvelle phénoménologie&quot; française, comme chez Levinas ou Marion, explorant l'expérience de la singularité, l'affectivité et les rapports entre monde fini et infini. Dans des ouvrages tels que Neue Phänomenologie in Frankreich (2012) ou Welt und Unendlichkeit (posthume, 2014), il questionne les fondements de la métaphysique  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Ph%C3%A9nom%C3%A9nologie_(philosophie)&quot;  title=&quot; Phénoménologie  par Wikipedia&quot;&gt;phénoménologique, &lt;/a&gt; sans aborder explicitement l'agnosticisme, mais en soulignant les horizons inconnaissables de l'expérience. &lt;/p&gt; &lt;p&gt; Bien qu'aucun lien direct n'apparaisse avec l'origine de  &lt;a href=&quot;https://fr.wikipedia.org/wiki/Agnosticisme&quot;  title=&quot; Agnosticisme  par Wikipedia&quot;&gt;l'agnosticisme &lt;/a&gt;  – forgé par Thomas Huxley en 1869 et remontant à Protagoras –, Tengelyi a contribué à des débats sur la connaissance et l'absolu via son engagement dans des revues comme Annales de phénoménologie. Un document mentionne &quot;di-agnostique Henry&quot; près de son nom, peut-être une référence contextuelle à des discussions philosophiques sur le doute épistémologique, mais cela reste marginal. &lt;/p&gt; &lt;p&gt; Il i reste une figure clé de la phénoménologie contemporaine européenne, avec des publications en hongrois, allemand et français, et un engagement public, comme sa lettre ouverte en 2011 défendant des intellectuels hongrois face à des attaques médiatiques. &lt;/p&gt; &#10;&#10;"/>
+    <hyperlink ref="H90" r:id="rId81" display="https://laphilo.fr/pho/ltengelyi-mini.webp"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>